<commit_message>
Populate CMC_ENS datasets and rebuild outputs pipeline
</commit_message>
<xml_diff>
--- a/outputs/historical_hdd_thresholds.xlsx
+++ b/outputs/historical_hdd_thresholds.xlsx
@@ -1210,7 +1210,7 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>-152</v>
+        <v>-160</v>
       </c>
       <c r="C13" s="10" t="n">
         <v>52</v>
@@ -1273,7 +1273,7 @@
         <v>-24</v>
       </c>
       <c r="W13" s="10" t="n">
-        <v>-152</v>
+        <v>-160</v>
       </c>
       <c r="X13" s="10" t="n">
         <v>106</v>
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C14" s="5" t="n">
         <v>86</v>

</xml_diff>

<commit_message>
feat: Multi-page UI pivot (Phase 1-4) with historical Chart.js visualizations
</commit_message>
<xml_diff>
--- a/outputs/historical_hdd_thresholds.xlsx
+++ b/outputs/historical_hdd_thresholds.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HDD Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HDD Matrix" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Phase 3: Implement frontend cache-busting and shift table display rules
</commit_message>
<xml_diff>
--- a/outputs/historical_hdd_thresholds.xlsx
+++ b/outputs/historical_hdd_thresholds.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HDD Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HDD Matrix" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1210,7 +1210,7 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>-303</v>
+        <v>-205</v>
       </c>
       <c r="C13" s="10" t="n">
         <v>52</v>
@@ -1273,7 +1273,7 @@
         <v>-24</v>
       </c>
       <c r="W13" s="10" t="n">
-        <v>-303</v>
+        <v>-205</v>
       </c>
       <c r="X13" s="10" t="n">
         <v>106</v>
@@ -1282,7 +1282,7 @@
         <v>4</v>
       </c>
       <c r="Z13" s="10" t="n">
-        <v>-11</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="14">
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C14" s="5" t="n">
         <v>86</v>

</xml_diff>

<commit_message>
fix: restore fully merged data tables and analytics dropdown
</commit_message>
<xml_diff>
--- a/outputs/historical_hdd_thresholds.xlsx
+++ b/outputs/historical_hdd_thresholds.xlsx
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>31</v>
@@ -1027,7 +1027,7 @@
         <v>31</v>
       </c>
       <c r="W8" s="5" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="X8" s="5" t="n">
         <v>31</v>
@@ -1046,7 +1046,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>151</v>
@@ -1109,7 +1109,7 @@
         <v>151</v>
       </c>
       <c r="W9" s="7" t="n">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="X9" s="7" t="n">
         <v>152</v>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1</v>
+        <v>0.9867549668874173</v>
       </c>
       <c r="C10" s="8" t="n">
         <v>1</v>
@@ -1191,7 +1191,7 @@
         <v>1</v>
       </c>
       <c r="W10" s="8" t="n">
-        <v>1</v>
+        <v>0.9867549668874173</v>
       </c>
       <c r="X10" s="8" t="n">
         <v>1.006622516556291</v>
@@ -1200,7 +1200,7 @@
         <v>1.001986754966887</v>
       </c>
       <c r="Z10" s="8" t="n">
-        <v>1.00157678965626</v>
+        <v>1.000946073793756</v>
       </c>
     </row>
     <row r="13">
@@ -1210,7 +1210,7 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>-75</v>
+        <v>-208</v>
       </c>
       <c r="C13" s="10" t="n">
         <v>52</v>
@@ -1273,7 +1273,7 @@
         <v>-24</v>
       </c>
       <c r="W13" s="10" t="n">
-        <v>-115</v>
+        <v>-208</v>
       </c>
       <c r="X13" s="10" t="n">
         <v>106</v>
@@ -1282,7 +1282,7 @@
         <v>4</v>
       </c>
       <c r="Z13" s="10" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="14">
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C14" s="5" t="n">
         <v>86</v>

</xml_diff>

<commit_message>
chore: push new map artifacts, model run CSVs, and chart outputs
</commit_message>
<xml_diff>
--- a/outputs/historical_hdd_thresholds.xlsx
+++ b/outputs/historical_hdd_thresholds.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HDD Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HDD Matrix" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Fix seasonal cumulative CDD curve bias by moving GRIB downloads to 6-hourly step resolution
</commit_message>
<xml_diff>
--- a/outputs/historical_hdd_thresholds.xlsx
+++ b/outputs/historical_hdd_thresholds.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HDD Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HDD Matrix" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>